<commit_message>
Preserve exact billing period answers
</commit_message>
<xml_diff>
--- a/artifacts/关键标准答案.xlsx
+++ b/artifacts/关键标准答案.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R2391e66c2eb743d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="R4f69346034e54f68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="R90695cc8a5e84d43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="R08f03a76068740b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="R2ac11b1a6dca40b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R9e92bd9285944ca7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="Ra595f541b4c84636"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="R4480807f1453426b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="R70c354687dc64098"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="Re0c8f1047d294d5b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -534,7 +534,7 @@
         <x:v>billing_meta.billing_period_start</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>2026年7月1日00:00:00Z</x:v>
+        <x:v>ISO8601值2026-07-01T00:00:00Z</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
         <x:v>billing_contract.json的billing_period_start_utc</x:v>
@@ -548,7 +548,7 @@
         <x:v>billing_meta.billing_period_end</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
-        <x:v>2026年8月1日00:00:00Z</x:v>
+        <x:v>ISO8601值2026-08-01T00:00:00Z</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
         <x:v>billing_contract.json的billing_period_end_utc</x:v>

</xml_diff>